<commit_message>
Linka 155: oprava textov v hre (gramatika, pravopis, štýl)
- Gramatika a pravopis: „políciu netreba“, „ho to koplo“, „predtým“,
  „zďaleka“, „zaparí“, „pokoj“ namiesto „kľud“, „odmalička“, „mame sa točí“,
  „dievča je opité“, „ochrnúť“ v správnom význame, „Warfarín“ jednotne,
  „Presná triáž“ namiesto neexistujúceho „triážnik“.
- Vety zlepené pomlčkou rozdelené na bodku, čiarku alebo dvojbodku
  (vysvetlenia zlých pokynov, tipy kurzu, kazuistiky, hlásenia, menu).
- Otázky operátora bez zápornej, sugestívnej formy.
- V rozbore je vysvetlenie chybného pokynu na samostatnom riadku.
- Scenár viet a Excel obnovené; nahrané vety ostali bez zmeny.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ShEd6fCg1yi4tRkJ1tRpTi
</commit_message>
<xml_diff>
--- a/dispecing/kontrola/Linka155-kontrola-obsahu.xlsx
+++ b/dispecing/kontrola/Linka155-kontrola-obsahu.xlsx
@@ -240,8 +240,8 @@
 • Neprestávajte, kým nepríde posádka, aj keď sa vám zdá, že to nepomáha.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Zatraste ním, aby sa prebral. – trasenie dojčaťa je nebezpečné a stráca čas – treba hneď stláčať a vdychovať.
-• Dajte mu napiť, nech sa preberie. – dojča bez vedomia nevie prehĺtať – voda mu zatečie do dýchacích ciest.</t>
+    <t xml:space="preserve">• Zatraste ním, aby sa prebral. – trasenie dojčaťa je nebezpečné a stráca čas. Treba hneď stláčať a vdychovať.
+• Dajte mu napiť, nech sa preberie. – dojča bez vedomia nevie prehĺtať a voda mu zatečie do dýchacích ciest.</t>
   </si>
   <si>
     <t xml:space="preserve">Nové: TANR dojčaťa – dva prsty, asi 4 cm, ak to volajúci vie, 5 vdychov do úst aj nosa a 15 : 2.</t>
@@ -258,7 +258,7 @@
     <t xml:space="preserve">Nereaguje… ani keď ho štipnem. Ale chrápe, takže spí, nie?</t>
   </si>
   <si>
-    <t xml:space="preserve">Áno, dýcha – tak nahlas chrápe, raz za čas.</t>
+    <t xml:space="preserve">Áno, dýcha… tak nahlas chrápe, raz za čas.</t>
   </si>
   <si>
     <t xml:space="preserve">Okolo úst je taký sivý.</t>
@@ -289,7 +289,7 @@
 • Ak je vás viac, každé dve minúty sa pri stláčaní vystriedajte.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Prestaňte na chvíľu stláčať a skúste mu nahmatať pulz. – každé prerušenie stláčania znižuje šancu na prežitie – stláča sa bez prestávky, kým nepríde posádka.
+    <t xml:space="preserve">• Prestaňte na chvíľu stláčať a skúste mu nahmatať pulz. – každé prerušenie stláčania znižuje šancu na prežitie. Stláča sa bez prestávky, kým nepríde posádka.
 • Dajte mu napiť vody, nech sa preberie. – človek bez vedomia nevie prehĺtať a voda mu zatečie do dýchacích ciest.</t>
   </si>
   <si>
@@ -300,7 +300,7 @@
 H3 · nie je pri ňom</t>
   </si>
   <si>
-    <t xml:space="preserve">„Volám z Nemecka – otec mi na videohovore spadol zo stoličky a nereaguje! Mama je doma s ním.“</t>
+    <t xml:space="preserve">„Volám z Nemecka. Otec mi na videohovore spadol zo stoličky a nereaguje! Mama je doma s ním.“</t>
   </si>
   <si>
     <t xml:space="preserve">Neviem, cez kameru nereagoval.</t>
@@ -525,10 +525,10 @@
 • Je tam ešte niekto, kto môže pomôcť? → Je tu so mnou babka.</t>
   </si>
   <si>
-    <t xml:space="preserve">Úmrtie doma – prehliadka mŕtveho tela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Podľa tvojej odpovede: doma pri dlho chorom bez podozrenia stačí prehliadka mŕtveho tela, polícia netreba.</t>
+    <t xml:space="preserve">Úmrtie doma: prehliadka mŕtveho tela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Podľa tvojej odpovede: doma pri dlho chorom bez podozrenia stačí prehliadka mŕtveho tela, políciu netreba.</t>
   </si>
   <si>
     <t xml:space="preserve">Mŕtvy na lavičke
@@ -563,7 +563,7 @@
 • Poznáte ho? → Nie, nikdy som ho nevidel.</t>
   </si>
   <si>
-    <t xml:space="preserve">Úmrtie na verejnosti alebo nejasné – prehliadka a polícia</t>
+    <t xml:space="preserve">Úmrtie na verejnosti alebo nejasné: prehliadka a polícia</t>
   </si>
   <si>
     <t xml:space="preserve">Nové podľa tvojej odpovede: úmrtie na verejnosti – prehliadka a polícia. Bez polície −20.</t>
@@ -638,15 +638,15 @@
 • Aké lieky berie? Vzal si ich dnes? → Neviem presne.
 • Koľko má rokov? → Asi sedemdesiat.
 • Stalo sa mu to už niekedy? → Neviem o tom.
-• Mal pred tým bolesť na hrudi alebo búšenie srdca? → Neviem, ráno nič nehovorila.</t>
+• Mal predtým bolesť na hrudi alebo búšenie srdca? → Neviem, ráno nič nehovorila.</t>
   </si>
   <si>
     <t xml:space="preserve">• Otočte ju na bok do stabilizovanej polohy a jemne jej zakloňte hlavu.
-• Ostaňte pri nej a sledujte dych – keby prestala dýchať, hneď mi to povedzte.</t>
+• Ostaňte pri nej a sledujte dych. Keby prestala dýchať, hneď mi to povedzte.</t>
   </si>
   <si>
     <t xml:space="preserve">• Dajte jej napiť, nech sa preberie. – v bezvedomí nevie prehĺtať a voda jej zatečie do dýchacích ciest.
-• Podložte jej hlavu vysokým vankúšom. – hlava ohnutá dopredu zatvorí dýchacie cesty – treba ju zakloniť a otočiť na bok.</t>
+• Podložte jej hlavu vysokým vankúšom. – hlava ohnutá dopredu zatvorí dýchacie cesty. Treba ju zakloniť a otočiť na bok.</t>
   </si>
   <si>
     <t xml:space="preserve">Opravené: odpoveď „dýcha pravidelne, len trochu chrápe“, v strome NZO ostali len lapavé dychy.</t>
@@ -690,8 +690,8 @@
 • Pripravte jeho glukomer a lieky pre záchranárov.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nalejte mu do úst sladký čaj. – človek v bezvedomí nevie prehĺtať – sladké sa dáva ústami len tomu, kto je pri vedomí.
-• Pichnite mu jeho inzulín. – spotený diabetik v bezvedomí má skôr nízky cukor – inzulín ho zníži ešte viac.</t>
+    <t xml:space="preserve">• Nalejte mu do úst sladký čaj. – človek v bezvedomí nevie prehĺtať. Sladké sa dáva ústami len tomu, kto je pri vedomí.
+• Pichnite mu jeho inzulín. – spotený diabetik v bezvedomí má skôr nízky cukor a inzulín ho zníži ešte viac.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (porucha vedomia K, nič ústami pri bezvedomí).</t>
@@ -726,14 +726,14 @@
 • Udrel si hlavu, stratil vedomie? → Trochu sa udrela do hlavy, keď padala.
 • ★ Aké lieky berie? Vzal si ich dnes? → Áno, Warfarín a niečo na tlak.
 • ★ Koľko má rokov? → Osemdesiatdva.
-• Mal pred tým bolesť na hrudi alebo búšenie srdca? → Pred tým hovorila, že jej je slabo.</t>
+• Mal predtým bolesť na hrudi alebo búšenie srdca? → Predtým hovorila, že jej je slabo.</t>
   </si>
   <si>
     <t xml:space="preserve">• Nech zostane sedieť alebo ležať, sama nevstáva.
 • Pripravte jej lieky a zdravotnú dokumentáciu.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Postavte ju, nech sa prejde. – po kolapse môže znova odpadnúť a pri páde sa zraniť – nech leží alebo sedí.</t>
+    <t xml:space="preserve">• Postavte ju, nech sa prejde. – po kolapse môže znova odpadnúť a pri páde sa zraniť. Nech leží alebo sedí.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N). Berie Warfarín a udrela si hlavu – nemala by byť K? Overiť.</t>
@@ -811,7 +811,7 @@
 • Aké lieky berie? Vzal si ich dnes? → Neviem, nešiel som k nemu.
 • Koľko má rokov? → Neviem, nešiel som k nemu.
 • Stalo sa mu to už niekedy? → Neviem, nešiel som k nemu.
-• Mal pred tým bolesť na hrudi alebo búšenie srdca? → Neviem, nešiel som k nemu.
+• Mal predtým bolesť na hrudi alebo búšenie srdca? → Neviem, nešiel som k nemu.
 • Môžete pri ňom počkať, kým niekto príde? → Nie, ponáhľam sa. Zbohom.
 • Dýcha? Videli ste, či sa hýbe? → Neviem, nešiel som k nemu.</t>
   </si>
@@ -857,7 +857,7 @@
 • ★ Stalo sa vám to už niekedy? → Áno, keď dlho stojím v teple.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rada volajúcemu – postup doma
+    <t xml:space="preserve">Rada volajúcemu: postup doma
 Odporučiť 116117 alebo všeobecného lekára</t>
   </si>
   <si>
@@ -890,14 +890,14 @@
 • ★ Mohol niečo vdýchnuť alebo prehltnúť? → Kus mäsa pri obede.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ak vie kašľať, nech silno kašle – nič iné nerobte.
+    <t xml:space="preserve">• Ak vie kašľať, nech silno kašle a nič iné nerobte.
 • Ak nevie kašľať, predkloňte ho a 5-krát ho udrite medzi lopatky.
 • Keď to nepomôže, 5-krát mu stlačte brucho pod rebrami dnu a hore.
 • Keby stratil vedomie, položte ho na zem a začnite stláčať hrudník.</t>
   </si>
   <si>
     <t xml:space="preserve">• Dajte mu napiť vody, nech to spláchne. – tekutina upchatými dýchacími cestami neprejde a upchá ich ešte viac.
-• Strčte mu prsty hlboko do krku a vytiahnite to. – vyberanie naslepo zatlačí predmet hlbšie – pomáhajú údery medzi lopatky a stláčanie brucha.</t>
+• Strčte mu prsty hlboko do krku a vytiahnite to. – vyberanie naslepo zatlačí predmet hlbšie. Pomáhajú údery medzi lopatky a stláčanie brucha.</t>
   </si>
   <si>
     <t xml:space="preserve">Doplnené: pokyn „Ak vie kašľať, nech silno kašle“.</t>
@@ -938,7 +938,7 @@
 • Otvorte okno a uvoľnite mu oblečenie.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Uložte ho do postele na chrbát. – v ľahu sa pri dýchavici dýcha horšie – nech sedí.</t>
+    <t xml:space="preserve">• Uložte ho do postele na chrbát. – v ľahu sa pri dýchavici dýcha horšie, preto nech sedí.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (cyanóza, nevie hovoriť = K).</t>
@@ -962,7 +962,7 @@
   <si>
     <t xml:space="preserve">• Kedy sa to začalo? Prišlo to náhle? → Asi pred pol hodinou.
 • ★ Vie povedať celú vetu? → Len dve-tri slová.
-• Má astmu alebo chronickú chorobu pľúc? → Áno, má astmu od malička.
+• Má astmu alebo chronickú chorobu pľúc? → Áno, má astmu odmalička.
 • ★ Má inhalátor alebo kyslík? Použil ho? → Štyri, nepomáha to.
 • Bolí ho pri tom na hrudi? → Nie, len nemôže dýchať.</t>
   </si>
@@ -1003,11 +1003,11 @@
 • ★ Bolí ho pri tom na hrudi? → Nie, hovorí, že nie.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Hovorte s ňou pokojne a nech dýcha pomaly – nádych nosom, pomalý výdych ústami.
+    <t xml:space="preserve">• Hovorte s ňou pokojne a nech dýcha pomaly: nádych nosom, pomalý výdych ústami.
 • Nech si sadne a uvoľní sa.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nech dýcha do igelitového vrecka. – dýchanie do vrecka je nebezpečné – môže chýbať kyslík, stačí pokojné pomalé dýchanie.</t>
+    <t xml:space="preserve">• Nech dýcha do igelitového vrecka. – dýchanie do vrecka je nebezpečné, lebo môže chýbať kyslík. Stačí pokojné pomalé dýchanie.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (M). Otázky vylučujú bolesť na hrudi.</t>
@@ -1043,7 +1043,7 @@
   </si>
   <si>
     <t xml:space="preserve">Odporučiť 116117 alebo všeobecného lekára
-Rada volajúcemu – postup doma</t>
+Rada volajúcemu: postup doma</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (O, 116117).</t>
@@ -1073,7 +1073,7 @@
 • Dajte jej studený obklad na zátylok.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nech si ľahne a zakloní hlavu. – pri zaklonení steká krv do hrdla a žalúdka – treba sa predkloniť.</t>
+    <t xml:space="preserve">• Nech si ľahne a zakloní hlavu. – pri zaklonení steká krv do hrdla a žalúdka. Treba sa predkloniť.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N – antikoagulancia, nedá sa zastaviť).</t>
@@ -1113,7 +1113,7 @@
 • Odfoťte zvratky pre záchranárov.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte mu vypiť mlieko na žalúdok. – pri krvácaní zo žalúdka nesmie nič piť – môže ísť na endoskopiu alebo operáciu.</t>
+    <t xml:space="preserve">• Dajte mu vypiť mlieko na žalúdok. – pri krvácaní zo žalúdka nesmie nič piť, lebo môže ísť na endoskopiu alebo operáciu.</t>
   </si>
   <si>
     <t xml:space="preserve">Zastavené krvácanie z nosa
@@ -1136,7 +1136,7 @@
 • Udrel sa do nosa? → Nie, len si ho šúchal.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rada volajúcemu – postup doma</t>
+    <t xml:space="preserve">Rada volajúcemu: postup doma</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (O).</t>
@@ -1162,8 +1162,8 @@
 • Pripravte si doklady a zoznam liekov, nech sú pri vás.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Skúste sa rozchodiť, nech sa chrbát uvoľní. – pri úniku moču a necitlivosti v rozkroku môže ísť o útlak nervov – chôdza hrozí pádom, nech leží.
-• Zoberte si tabletku proti bolesti a uvidíme. – operátor po telefóne lieky neodporúča – o liečbe rozhodne posádka.</t>
+    <t xml:space="preserve">• Skúste sa rozchodiť, nech sa chrbát uvoľní. – pri úniku moču a necitlivosti v rozkroku môže ísť o útlak nervov. Chôdza hrozí pádom, nech leží.
+• Zoberte si tabletku proti bolesti a uvidíme. – operátor po telefóne lieky neodporúča, o liečbe rozhodne posádka.</t>
   </si>
   <si>
     <t xml:space="preserve">Nové podľa tvojej odpovede: úvodná veta je podobná ako pri M, N až keď doplňujúce otázky odhalia únik moču a necitlivosť v rozkroku.</t>
@@ -1192,7 +1192,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Dajte mu na brucho termofor. – teplo pri náhlej bolesti brucha môže zhoršiť zápal, napríklad slepého čreva.
-• Dajte mu silný liek proti bolesti. – liek môže zakryť príznaky a pacient môže ísť na operáciu – nesmie nič ústami.</t>
+• Dajte mu silný liek proti bolesti. – liek môže zakryť príznaky a pacient môže ísť na operáciu. Nesmie nič ústami.</t>
   </si>
   <si>
     <t xml:space="preserve">Studená noha
@@ -1298,9 +1298,9 @@
 • Pripravte jeho lieky a odomknite dvere pre záchranku.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ak nie je alergický na aspirín, nech jednu tabletu rozhryzie. – operátor po telefóne lieky neodporúča – o liečbe rozhodne posádka.
-• Nech sa prejde, možno to rozchodí. – námaha pri infarkte zväčšuje poškodenie srdca – nech sedí v pokoji.
-• Odvezte ho radšej sami autom do nemocnice. – srdce môže kedykoľvek zlyhať a v aute mu nikto nepomôže – nech čaká na záchranku.</t>
+    <t xml:space="preserve">• Ak nie je alergický na aspirín, nech jednu tabletu rozhryzie. – operátor po telefóne lieky neodporúča, o liečbe rozhodne posádka.
+• Nech sa prejde, možno to rozchodí. – námaha pri infarkte zväčšuje poškodenie srdca, preto nech sedí v pokoji.
+• Odvezte ho radšej sami autom do nemocnice. – srdce môže kedykoľvek zlyhať a v aute mu nikto nepomôže. Nech čaká na záchranku.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (K). Opravené: aspirín je chybný pokyn – po telefóne sa nepodáva.</t>
@@ -1336,8 +1336,8 @@
 • Oblečte ho do suchého a prikryte, nech neprechladne.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ak nie je alergický na aspirín a máte ho, nech jednu tabletu rozhryzie. – operátor po telefóne lieky neodporúča – o liečbe rozhodne posádka.
-• Nech pomaly pokračuje k najbližšej chate. – námaha pri bolesti na hrudi môže spôsobiť zástavu srdca – nech čaká na mieste.
+    <t xml:space="preserve">• Ak nie je alergický na aspirín a máte ho, nech jednu tabletu rozhryzie. – operátor po telefóne lieky neodporúča, o liečbe rozhodne posádka.
+• Nech pomaly pokračuje k najbližšej chate. – námaha pri bolesti na hrudi môže spôsobiť zástavu srdca. Nech čaká na mieste.
 • Dajte mu glg slivovice na zahriatie. – alkohol rozšíri cievy, telo rýchlejšie stráca teplo a srdce sa viac zaťaží.</t>
   </si>
   <si>
@@ -1378,17 +1378,17 @@
 • Kedy sa to začalo? Prišlo to náhle? → Asi pred štyridsiatimi minútami.
 • Lieči sa so srdcom? Mal infarkt alebo stent? → Nie, so srdcom som sa neliečil.
 • Aké lieky berie? Vzal si ich dnes? → Len na tlak.
-• Má aj iné ťažkosti – poruchu reči, slabú ruku, zle vidí? → Nie.
+• Má aj iné ťažkosti, napríklad poruchu reči, slabú ruku alebo zle vidí? → Nie.
 • Odpadol, stratil vedomie? → Nie.
 • Koľko má rokov? → Šesťdesiatjeden.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Sadnite si alebo si polosadnite a nenamáhajte sa.
+    <t xml:space="preserve">• Sadnite si alebo sa uložte do polosedu a nenamáhajte sa.
 • Ak to zvládnete, odomknite dvere a znova si sadnite.
 • Pripravte si zoznam liekov.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Prejdite sa po byte, nech sa to rozchodí. – pri bolesti na hrudi treba pokoj – námaha zvyšuje nárok srdca na kyslík.</t>
+    <t xml:space="preserve">• Prejdite sa po byte, nech sa to rozchodí. – pri bolesti na hrudi treba pokoj, lebo námaha zvyšuje nárok srdca na kyslík.</t>
   </si>
   <si>
     <t xml:space="preserve">Nové (skryté H3): z pamäti volajúcej to vyzerá na N, pacient po zavolaní späť má K.</t>
@@ -1417,7 +1417,7 @@
 • Koľko máte pulz? Bije srdce pravidelne? → Neviem, srdce mi búši.
 • Liečite sa so srdcom? Mali ste infarkt alebo stent? → Nie, liečim sa len s cukrovkou a tlakom.
 • Aké lieky beriete? Vzali ste si ich dnes? → Na cukrovku a na tlak.
-• Máte aj iné ťažkosti – poruchu reči, slabú ruku, zle vidíte? → Nie, len je mi strašne slabo.
+• Máte aj iné ťažkosti, napríklad poruchu reči, slabú ruku alebo zle vidíte? → Nie, len je mi strašne slabo.
 • Odpadli ste? → Nie, ale točí sa mi hlava.
 • Koľko máte rokov? → Päťdesiatosem.</t>
   </si>
@@ -1427,8 +1427,8 @@
 • Ak vám bude horšie alebo budete omdlievať, hneď volajte znova.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Prejdite sa na čerstvom vzduchu, možno to prejde. – pri podozrení na infarkt každá námaha zaťažuje srdce – pacient má byť v pokoji.
-• Vezmite si niečo na žalúdok a ľahnite si. – pálenie so studeným potom a dýchavicou môže byť infarkt – liek na žalúdok nepomôže a stráca sa čas.</t>
+    <t xml:space="preserve">• Prejdite sa na čerstvom vzduchu, možno to prejde. – pri podozrení na infarkt každá námaha zaťažuje srdce. Pacient má byť v pokoji.
+• Vezmite si niečo na žalúdok a ľahnite si. – pálenie so studeným potom a dýchavicou môže byť infarkt. Liek na žalúdok nepomôže a stráca sa čas.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: netypický infarkt u ženy (H1) – pálenie pod hrudnou kosťou, vyžarovanie, studený pot, dýchavica – K. Overiť, či K alebo N.</t>
@@ -1438,7 +1438,7 @@
 H2 · pri ňom</t>
   </si>
   <si>
-    <t xml:space="preserve">„Otec má v hrudi defibrilátor a už trikrát ho to strašne kopla!“</t>
+    <t xml:space="preserve">„Otec má v hrudi defibrilátor a už trikrát ho to strašne koplo!“</t>
   </si>
   <si>
     <t xml:space="preserve">Je zmätený, nevie, čo sa deje.</t>
@@ -1449,7 +1449,7 @@
 • Lieči sa so srdcom? Mal infarkt alebo stent? → Áno, má defibrilátor pre zlé srdce.
 • Aké lieky berie? Vzal si ich dnes? → Berie lieky na srdce.
 • ★ Odpadol, stratil vedomie? → Na chvíľu áno, pri prvom výboji.
-• Koľkokrát ho to kopla? → Trikrát za desať minút.</t>
+• Koľkokrát ho to koplo? → Trikrát za desať minút.</t>
   </si>
   <si>
     <t xml:space="preserve">• Nech leží alebo sedí v pokoji.
@@ -1500,7 +1500,7 @@
     <t xml:space="preserve">„Mama mi ráno volala, že ju tlačí na hrudi, a teraz mi nedvíha telefón. Býva sama a ja som v Bratislave.“</t>
   </si>
   <si>
-    <t xml:space="preserve">Neviem, nie som pri nej – nedvíha telefón.</t>
+    <t xml:space="preserve">Neviem, nie som pri nej. Nedvíha telefón.</t>
   </si>
   <si>
     <t xml:space="preserve">To neviem, nie som tam.</t>
@@ -1575,7 +1575,7 @@
 • Kedy sa to začalo? Prišlo to náhle? → Asi hodinu.
 • Koľko ukazuje tlakomer? → 180 na 100.
 • ★ Aké lieky beriete? Vzali ste si ich dnes? → Áno, ale dnes som ich zabudla.
-• ★ Máte aj iné ťažkosti – poruchu reči, slabú ruku, zle vidíte? → Nie, len ma trochu bolí hlava.</t>
+• ★ Máte aj iné ťažkosti, napríklad poruchu reči, slabú ruku alebo zle vidíte? → Nie, len ma trochu bolí hlava.</t>
   </si>
   <si>
     <t xml:space="preserve">Nové: tlak 180/100 s miernou bolesťou hlavy – M podľa stromu kardio.</t>
@@ -1642,7 +1642,7 @@
 • Pozrite sa na hodinky a merajte, ako dlho záchvat trvá.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vložte mu do úst lyžicu, nech si neodhryzne jazyk. – do úst sa pri kŕčoch nič nevkladá – hrozí poranenie a vdýchnutie.
+    <t xml:space="preserve">• Vložte mu do úst lyžicu, nech si neodhryzne jazyk. – do úst sa pri kŕčoch nič nevkladá, hrozí poranenie a vdýchnutie.
 • Pevne ho držte, nech sa netrasie. – násilné držanie kŕče nezastaví a hrozí poranenie.</t>
   </si>
   <si>
@@ -1686,8 +1686,8 @@
 • Ak bude zvracať alebo prestane reagovať, otočte ju na bok a hneď volajte.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte jej vypiť kávu, nech sa preberie. – pri mozgovej príhode môže byť porušené prehĺtanie – nič ústami.
-• Nech si ľahne a vyspí sa, ráno sa uvidí. – pri mozgovej príhode rozhoduje čas – liečba je možná len niekoľko hodín od začiatku.</t>
+    <t xml:space="preserve">• Dajte jej vypiť kávu, nech sa preberie. – pri mozgovej príhode môže byť porušené prehĺtanie, preto nič ústami.
+• Nech si ľahne a vyspí sa, ráno sa uvidí. – pri mozgovej príhode rozhoduje čas: liečba je možná len niekoľko hodín od začiatku.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: FAST, čas „naposledy v poriadku“, riedenie krvi – N. Chyták: volajúca chce čakať do rána.</t>
@@ -1720,7 +1720,7 @@
 • Vyzlečte ju do ľahkého a neprikrývajte ju.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte ju do studenej vane. – studený kúpeľ je pre telo šok – stačí ľahké oblečenie.</t>
+    <t xml:space="preserve">• Dajte ju do studenej vane. – studený kúpeľ je pre telo šok. Stačí ľahké oblečenie.</t>
   </si>
   <si>
     <t xml:space="preserve">Kamarátka napísala, že nevie hovoriť
@@ -1767,7 +1767,7 @@
   <si>
     <t xml:space="preserve">• ★ Kedy sa to začalo? Prišlo to náhle? → Pred dvadsiatimi minútami, pri obede bola ešte v poriadku.
 • Ovisol mu kútik, má slabú ruku alebo poruchu reči? → Áno, ovisol jej kútik a nevie poriadne hovoriť.
-• ★ Berie lieky na riedenie krvi? → Áno, berie Warfarin.
+• ★ Berie lieky na riedenie krvi? → Áno, berie Warfarín.
 • Koľko má rokov? → Sedemdesiatštyri.</t>
   </si>
   <si>
@@ -1777,7 +1777,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Dajte jej aspirín, rozriedi krv. – pri porážke nesmie dostať nič ústami, a ak krváca do mozgu, aspirín to zhorší.
-• Nechajte ju vyspať, ráno to bude lepšie. – pri mozgovej príhode rozhoduje čas – liečba musí začať čo najskôr.</t>
+• Nechajte ju vyspať, ráno to bude lepšie. – pri mozgovej príhode rozhoduje čas: liečba musí začať čo najskôr.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N podľa stromu). Otázka na čas začiatku je, BE-FAST čiastočne.</t>
@@ -1844,7 +1844,7 @@
 • Keď príde polícia, povedzte im, kde je a čo má v ruke.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Choďte ho upokojiť, vás počúvne. – agresívny človek s nožom ohrozuje aj blízkych – bezpečnosť má prednosť, rieši to polícia.</t>
+    <t xml:space="preserve">• Choďte ho upokojiť, vás počúvne. – agresívny človek s nožom ohrozuje aj blízkych. Bezpečnosť má prednosť, rieši to polícia.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N, PZ).</t>
@@ -1883,7 +1883,7 @@
 • Nechoďte k nemu nasilu, počkajte na pomoc.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Povedzte mu, nech nerobí scény, a choďte ho stiahnuť. – nátlak a náhly pohyb môžu človeka v kríze vyprovokovať – rozhovor a čakanie na pomoc sú bezpečnejšie.</t>
+    <t xml:space="preserve">• Povedzte mu, nech nerobí scény, a choďte ho stiahnuť. – nátlak a náhly pohyb môžu človeka v kríze vyprovokovať. Rozhovor a čakanie na pomoc sú bezpečnejšie.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N, PZ a HaZZ).</t>
@@ -1962,7 +1962,7 @@
 • Ak prestane dýchať, hneď mi to povedzte, začneme oživovať.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nech sa poprechádza na čerstvom vzduchu. – pri anafylaxii môže postavenie a chôdza spôsobiť náhly kolaps – nech sedí alebo leží.
+    <t xml:space="preserve">• Nech sa poprechádza na čerstvom vzduchu. – pri anafylaxii môže postavenie a chôdza spôsobiť náhly kolaps, preto nech sedí alebo leží.
 • Dajte jej vypiť mlieko, to zmierni opuch. – opuchnuté hrdlo nezvládne prehĺtanie a mlieko pri alergii nepomáha.</t>
   </si>
   <si>
@@ -2002,7 +2002,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Choďte sa napiť studenej vody, opuch splaskne. – pri anafylaxii hrozí pri postavení kolaps a opuchnuté hrdlo prehĺtanie nezvládne.
-• S perom počkajte, kým príde záchranka. – adrenalín treba pri anafylaxii podať hneď – každá minúta zhoršuje opuch dýchacích ciest.</t>
+• S perom počkajte, kým príde záchranka. – adrenalín treba pri anafylaxii podať hneď. Každá minúta zhoršuje opuch dýchacích ciest.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: anafylaxia (H1), opuch pier a jazyka, chrapot – N, navigovať adrenalínové pero.</t>
@@ -2082,8 +2082,8 @@
 • Keby prestal reagovať, nedávajte mu nič do úst a uložte ho na bok.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pichnite mu ešte inzulín, cukor mu určite stúpol. – pri nízkom cukre inzulín cukor ďalej zníži – hrozí bezvedomie a kŕče.
-• Nalejte mu do úst sladkú vodu, aj keď nereaguje. – kto nereaguje, nevie prehĺtať – tekutina zatečie do dýchacích ciest.</t>
+    <t xml:space="preserve">• Pichnite mu ešte inzulín, cukor mu určite stúpol. – pri nízkom cukre inzulín cukor ďalej zníži a hrozí bezvedomie a kŕče.
+• Nalejte mu do úst sladkú vodu, aj keď nereaguje. – kto nereaguje, nevie prehĺtať a tekutina mu zatečie do dýchacích ciest.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: hypoglykémia ako „porážka“ – glukomer 2,1, inzulín bez obeda, prehĺta – N (aj pri kategórii Neuro či Vedomie).</t>
@@ -2117,7 +2117,7 @@
 • Zmerajte mu cukor, ak máte glukomer.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pichnite mu inzulín. – zmätený a spotený diabetik má skôr nízky cukor – inzulín ho zníži ešte viac.</t>
+    <t xml:space="preserve">• Pichnite mu inzulín. – zmätený a spotený diabetik má skôr nízky cukor a inzulín ho zníži ešte viac.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N). Sladké len ak vie prehĺtať – je.</t>
@@ -2150,7 +2150,7 @@
 • O pätnásť minút si cukor zmerajte znova.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pichnite si inzulín, nech sa to vyrovná. – pri nízkom cukre inzulín cukor ešte zníži – môže prísť bezvedomie.</t>
+    <t xml:space="preserve">• Pichnite si inzulín, nech sa to vyrovná. – pri nízkom cukre inzulín cukor ešte zníži a môže prísť bezvedomie.</t>
   </si>
   <si>
     <t xml:space="preserve">Vysoký cukor bez ťažkostí
@@ -2199,7 +2199,7 @@
 • ★ Horí niečo alebo vyteká z auta? → Nie, nehorí, len sa z autobusu parí.
 • Ako sa to stalo, akou rýchlosťou? → Autobus narazil do auta a zišiel do priekopy.
 • Hýbe rukami aj nohami, cíti ich? → Neviem, nemôžem ku všetkým.
-• Kde presne je – v aute, na ceste, mimo cesty? → Autobus je v priekope, auto na ceste.
+• Kde presne je? V aute, na ceste, mimo cesty? → Autobus je v priekope, auto na ceste.
 • Ostal vodič na mieste? → Áno, šofér autobusu je tu.</t>
   </si>
   <si>
@@ -2214,8 +2214,8 @@
 • Krvácajúce rany stlačte čistou látkou.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Všetkých zranených povyťahujte z áut a uložte vedľa cesty. – vyťahovanie bez dôvodu môže zhoršiť poranenie chrbtice – von iba pri požiari alebo inom priamom nebezpečenstve.
-• Choďte doprostred cesty a mávajte na autá. – na ceste ohrozujete seba aj ostatných – zostaňte za zvodidlami a použite výstražné svetlá a trojuholník.</t>
+    <t xml:space="preserve">• Všetkých zranených povyťahujte z áut a uložte vedľa cesty. – vyťahovanie bez dôvodu môže zhoršiť poranenie chrbtice. Von ich ťahajte iba pri požiari alebo inom priamom nebezpečenstve.
+• Choďte doprostred cesty a mávajte na autá. – na ceste ohrozujete seba aj ostatných. Zostaňte za zvodidlami a použite výstražné svetlá a trojuholník.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (K). Na obrazovke OS je samostatné tlačidlo UHPO – zvážiť osobitný postup.</t>
@@ -2250,7 +2250,7 @@
     <t xml:space="preserve">• Koľko je zranených? → Jedna, tá pani.
 • Ako sa to stalo, akou rýchlosťou? → Asi päťdesiatkou, odletela niekoľko metrov.
 • Hýbe rukami aj nohami, cíti ich? → Neviem, len stoná.
-• ★ Kde presne je – v aute, na ceste, mimo cesty? → V jazdnom pruhu, autá ju obchádzajú.
+• ★ Kde presne je? V aute, na ceste, mimo cesty? → V jazdnom pruhu, autá ju obchádzajú.
 • ★ Ostal vodič na mieste? → Áno, stojí pri nej celý bledý.</t>
   </si>
   <si>
@@ -2258,8 +2258,8 @@
 • Zabezpečte miesto výstražnými svetlami, nech do nej nikto nenarazí.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Zdvihnite ju a posaďte na lavičku. – po zrazení autom môže mať poranenú chrbticu alebo vnútorné krvácanie – nehýbte s ňou.
-• Dajte jej napiť a niečo proti bolesti. – zranená nesmie nič piť ani brať lieky – môže ísť na operáciu.</t>
+    <t xml:space="preserve">• Zdvihnite ju a posaďte na lavičku. – po zrazení autom môže mať poranenú chrbticu alebo vnútorné krvácanie, preto s ňou nehýbte.
+• Dajte jej napiť a niečo proti bolesti. – zranená nesmie nič piť ani brať lieky, lebo môže ísť na operáciu.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (K, PZ).</t>
@@ -2293,7 +2293,7 @@
 • Horí niečo alebo vyteká z auta? → Nie, len z motorky kvapká benzín.
 • ★ Ako sa to stalo, akou rýchlosťou? → Išiel rýchlo, aspoň osemdesiat, vyletel zo sedla.
 • ★ Hýbe rukami aj nohami, cíti ich? → Rukami hýbe, ľavou nohou nie, vraví, že ho bolí.
-• ★ Kde presne je – v aute, na ceste, mimo cesty? → V priekope vedľa cesty, prilbu má na hlave.
+• ★ Kde presne je? V aute, na ceste, mimo cesty? → V priekope vedľa cesty, prilbu má na hlave.
 • Ostal vodič na mieste? → Áno, je tu.</t>
   </si>
   <si>
@@ -2302,11 +2302,11 @@
   <si>
     <t xml:space="preserve">• Prilbu mu nesnímajte, kým dýcha, a nech hýbe hlavou čo najmenej.
 • Krvácajúcu ranu na nohe stlačte čistou látkou a nepúšťajte.
-• Prikryte ho a zabezpečte miesto – výstražný trojuholník a svetlá.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Zložte mu prilbu, nech sa mu lepšie dýcha. – pri úraze hlavy a krku hrozí poškodenie miechy – prilba sa sníma len pri zastavenom dýchaní.
-• Pomôžte mu sadnúť si a vyrovnajte mu nohu. – zranený po páde z motorky môže mať poranenú chrbticu a zlomeninu – nehýbať ním.</t>
+• Prikryte ho a zabezpečte miesto výstražným trojuholníkom a svetlami.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Zložte mu prilbu, nech sa mu lepšie dýcha. – pri úraze hlavy a krku hrozí poškodenie miechy. Prilba sa sníma len pri zastavenom dýchaní.
+• Pomôžte mu sadnúť si a vyrovnajte mu nohu. – zranený po páde z motorky môže mať poranenú chrbticu a zlomeninu, preto s ním nehýbte.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: vymrštený motorkár, zmätený, deformita nohy – N, PZ, vrtuľník zvážiť, prilbu nesnímať.</t>
@@ -2334,7 +2334,7 @@
     <t xml:space="preserve">• Koľko je zranených? → Len motorkár.
 • ★ Ako sa to stalo, akou rýchlosťou? → Rýchlo, aspoň osemdesiatkou.
 • ★ Hýbe rukami aj nohami, cíti ich? → Rukami áno, ľavou nohou nie.
-• Kde presne je – v aute, na ceste, mimo cesty? → Leží za zvodidlami pri ceste.
+• Kde presne je? V aute, na ceste, mimo cesty? → Leží za zvodidlami pri ceste.
 • Ostal vodič na mieste? → Bol sám.</t>
   </si>
   <si>
@@ -2343,7 +2343,7 @@
 • Krvácajúcu ranu stlačte čistou látkou.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Posaďte ho a dajte mu napiť. – po náraze môže mať poranenú chrbticu aj vnútorné krvácanie – nehýbať a nič nepiť.</t>
+    <t xml:space="preserve">• Posaďte ho a dajte mu napiť. – po náraze môže mať poranenú chrbticu aj vnútorné krvácanie. Nehýbať s ním a nič nepiť.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N, PZ). Vrtuľník je v hre označený ako indikovaný (ťažký úraz) – overiť.</t>
@@ -2370,7 +2370,7 @@
 • Horí niečo alebo vyteká z auta? → Z motora sa trochu dymí.
 • Ako sa to stalo, akou rýchlosťou? → Narazil do stromu, auto je celé pokrčené.
 • Hýbe rukami aj nohami, cíti ich? → Rukami hýbe, nohu má zaseknutú.
-• ★ Kde presne je – v aute, na ceste, mimo cesty? → Na kolesách, prednou časťou v strome.
+• ★ Kde presne je? V aute, na ceste, mimo cesty? → Na kolesách, prednou časťou v strome.
 • Ostal vodič na mieste? → Je to on, iné auto tu nie je.
 • Je vodič pri vedomí a dýcha? → Je pri vedomí, stoná a krváca z nohy.</t>
   </si>
@@ -2380,8 +2380,8 @@
 • Krvácajúcu ranu stlačte čistou látkou.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vytiahnite ho z auta, kým nepríde pomoc. – zakliesneného vodiča môže vyťahovanie ochrnúť – vyslobodia ho hasiči so zdravotníkmi, von len pri požiari.
-• Dajte mu napiť, nech sa upokojí. – ťažko zranený pôjde možno na operáciu – nesmie piť.</t>
+    <t xml:space="preserve">• Vytiahnite ho z auta, kým nepríde pomoc. – zakliesnený vodič môže pri vyťahovaní ochrnúť. Vyslobodia ho hasiči so zdravotníkmi, von ho ťahajte len pri požiari.
+• Dajte mu napiť, nech sa upokojí. – ťažko zranený pôjde možno na operáciu, preto nesmie piť.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N, HaZZ a PZ).</t>
@@ -2400,7 +2400,7 @@
     <t xml:space="preserve">• ★ Koľko je zranených? → Nie, len ona.
 • Ako sa to stalo, akou rýchlosťou? → Nie veľmi rýchlo, zozadu.
 • Hýbe rukami aj nohami, cíti ich? → Áno, hýbe, len ju bolí krk.
-• Kde presne je – v aute, na ceste, mimo cesty? → Sedí v aute na kraji cesty.
+• Kde presne je? V aute, na ceste, mimo cesty? → Sedí v aute na kraji cesty.
 • Ostal vodič na mieste? → Áno, sme tu všetci.
 • Mravčia jej ruky? → Nie, len ju bolí krk.</t>
   </si>
@@ -2409,7 +2409,7 @@
 • Zapnite výstražné svetlá a postavte trojuholník.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nech si krk rozhýbe, to prejde. – pri bolesti krku po náraze môže byť poranená chrbtica – nehýbať.</t>
+    <t xml:space="preserve">• Nech si krk rozhýbe, to prejde. – pri bolesti krku po náraze môže byť poranená chrbtica, preto nehýbať hlavou.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (M, PZ – polícia ide k dopravným nehodám).</t>
@@ -2476,7 +2476,7 @@
     <t xml:space="preserve">Leží na chodníku pred barom. Útočník ušiel smerom k stanici.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Niekto ho bodol nožom.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Niekto ho bodol nožom.
 • ★ Kde presne je zranený? → V bruchu, vľavo.
 • Berie lieky na riedenie krvi? → Neviem, nepoznám ho.
 • Koľko má rokov? → Mladý, okolo dvadsaťpäť.
@@ -2489,8 +2489,8 @@
 • Nech leží a nehýbe sa.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Bežte za útočníkom a zadržte ho. – prenasledovať ozbrojeného útočníka je nebezpečné – zapamätajte si, kam utiekol, zvyšok urobí polícia.
-• Dajte mu napiť alkoholu na bolesť. – alkohol zhoršuje krvácanie a zranený nesmie piť – môže ísť na operáciu.</t>
+    <t xml:space="preserve">• Bežte za útočníkom a zadržte ho. – prenasledovať ozbrojeného útočníka je nebezpečné. Zapamätajte si, kam utiekol, zvyšok urobí polícia.
+• Dajte mu napiť alkoholu na bolesť. – alkohol zhoršuje krvácanie a zranený nesmie piť, lebo môže ísť na operáciu.</t>
   </si>
   <si>
     <t xml:space="preserve">Pád z lešenia
@@ -2512,7 +2512,7 @@
     <t xml:space="preserve">Leží na stavenisku, brána je otvorená.</t>
   </si>
   <si>
-    <t xml:space="preserve">• ★ Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Z tretieho poschodia, aspoň osem metrov.
+    <t xml:space="preserve">• ★ Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Z tretieho poschodia, aspoň osem metrov.
 • Udrel si hlavu, stratil vedomie? → Krváca z hlavy a neodpovedá.
 • ★ Hýbe rukami aj nohami, cíti ich? → Je pri vedomí, ale nohami nehýbe.
 • Kde presne je zranený? → Hlava a asi chrbát.
@@ -2525,7 +2525,7 @@
 • Sledujte, či dýcha, a keby prestal, hneď mi to povedzte.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Skúste ho posadiť a dať mu napiť. – po páde z výšky môže mať poranenú chrbticu a pohyb ho môže ochrnúť.
+    <t xml:space="preserve">• Skúste ho posadiť a dať mu napiť. – po páde z výšky môže mať poranenú chrbticu a pri pohybe môže ochrnúť.
 • Preneste ho do tieňa alebo dnu. – zraneného po páde sa presúva iba vtedy, keď mu hrozí bezprostredné nebezpečenstvo.</t>
   </si>
   <si>
@@ -2554,7 +2554,7 @@
     <t xml:space="preserve">Sme na dvore za domom.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Píla mu skĺzla do stehna.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Píla mu skĺzla do stehna.
 • Kde presne je zranený? → Stehno.
 • Koľko má rokov? → Päťdesiat.
 • ★ Je tam ešte niekto, kto môže pomôcť? → Áno, sused.
@@ -2566,8 +2566,8 @@
 • Nech leží a prikryte ho.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte mu vypiť pohár vody, stratil veľa tekutín. – ťažko zranený pôjde na operáciu – nesmie piť.
-• Ranu vypláchnite pod tečúcou vodou. – vyplachovanie zdrží zastavenie krvácania – tlak na ranu je najdôležitejší.</t>
+    <t xml:space="preserve">• Dajte mu vypiť pohár vody, stratil veľa tekutín. – ťažko zranený pôjde na operáciu, preto nesmie piť.
+• Ranu vypláchnite pod tečúcou vodou. – vyplachovanie zdrží zastavenie krvácania. Najdôležitejší je tlak na ranu.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (K). Tlak na ranu a turniket nad ranu – podľa skriptu.</t>
@@ -2592,7 +2592,7 @@
     <t xml:space="preserve">Leží na pláži, nehýbeme s ním.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Skočil šípku do plytkej vody.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Skočil šípku do plytkej vody.
 • Udrel si hlavu, stratil vedomie? → Udrel sa hlavou o dno, má odreté čelo.
 • ★ Hýbe rukami aj nohami, cíti ich? → Rukami trochu hýbe, nohami vôbec.
 • Kde presne je zranený? → Krk a hlava.
@@ -2601,7 +2601,7 @@
 • Ako dlho bol vo vode? → Hneď sme ho vytiahli.</t>
   </si>
   <si>
-    <t xml:space="preserve">podozrenie na poranenie chrbtice – šetrný a rýchly prevoz na neurochirurgiu</t>
+    <t xml:space="preserve">podozrenie na poranenie chrbtice, šetrný a rýchly prevoz na neurochirurgiu</t>
   </si>
   <si>
     <t xml:space="preserve">neurochirurgia</t>
@@ -2627,7 +2627,7 @@
     <t xml:space="preserve">Pošmykla sa na koberci a spadla na bok. Noha je nejaká kratšia a vytočená.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Pošmykla sa na koberci.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Pošmykla sa na koberci.
 • ★ Udrel si hlavu, stratil vedomie? → Je pri vedomí, rozpráva, len je trochu zmätená.
 • Hýbe rukami aj nohami, cíti ich? → Rukami áno, pravú nohu nedokáže zdvihnúť.
 • Kde presne je zranený? → Bok a noha.
@@ -2639,8 +2639,8 @@
 • Prikryte ju dekou, nech neprechladne.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Postavte ju na nohy, nech to rozchodí. – po páde môže mať zlomený krčok – na nohu sa nesmie postaviť.
-• Dajte jej niečo zo svojich liekov na tlak alebo na bolesť. – cudzie lieky môžu spôsobiť pád tlaku alebo sa pobiť s jeho liekmi.</t>
+    <t xml:space="preserve">• Postavte ju na nohy, nech to rozchodí. – po páde môže mať zlomený krčok, preto sa na nohu nesmie postaviť.
+• Dajte jej niečo zo svojich liekov na tlak alebo na bolesť. – cudzie lieky môžu spôsobiť pád tlaku alebo reagovať s liekmi, ktoré berie.</t>
   </si>
   <si>
     <t xml:space="preserve">Sused počul pád
@@ -2668,7 +2668,7 @@
 • ★ Koľko má rokov? → Asi osemdesiat.
 • ★ Je tam ešte niekto, kto môže pomôcť? → Je sám, nikoho nemá.
 • Po zavolaní späť: „Haló… spadol som v kúpeľni a neviem vstať.“
-• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Pošmykol som sa vo vani.
+• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Pošmykol som sa vo vani.
 • Udrel si hlavu, stratil vedomie? → Nie, hlavu som si neudrel.
 • Hýbe rukami aj nohami, cíti ich? → Rukami áno, pravú nohu nemôžem zdvihnúť.
 • Kde presne je zranený? → Pravé bedro.
@@ -2681,7 +2681,7 @@
 • Prikryte sa uterákom alebo čímkoľvek, nech vám nie je zima.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Skúste sa postaviť a dôjsť k dverám. – pri podozrení na zlomeninu bedra sa nemá postavovať – hrozí ďalší pád.</t>
+    <t xml:space="preserve">• Skúste sa postaviť a dôjsť k dverám. – pri podozrení na zlomeninu bedra sa nemá stavať na nohy, hrozí ďalší pád.</t>
   </si>
   <si>
     <t xml:space="preserve">Nové (H3): po zavolaní susedovi (H1) zistíš pád seniora s Warfarínom – M, hasiči na otvorenie.</t>
@@ -2700,7 +2700,7 @@
     <t xml:space="preserve">Nie, len je odretý.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Spadol z bicykla na ruku.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Spadol z bicykla na ruku.
 • ★ Udrel si hlavu, stratil vedomie? → Prilbu mal, hlavu si neudrel.
 • Hýbe rukami aj nohami, cíti ich? → Prstami hýbe, rukou nechce.
 • Kde presne je zranený? → Ľavá ruka, je krivá.
@@ -2727,7 +2727,7 @@
     <t xml:space="preserve">Sme na chodníku v lese, autom sa sem nedá. Do doliny je to asi hodinu.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Pošmykol sa na kameňoch.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Pošmykol sa na kameňoch.
 • ★ Hýbe rukami aj nohami, cíti ich? → Nemôže, noha je čudne vytočená, nekrváca.
 • Kde presne je zranený? → Pravý členok.
 • Koľko má rokov? → Tridsať.
@@ -2740,7 +2740,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Nech skúsi zísť dole aspoň k chate. – chôdza na zlomenej nohe poškodí cievy a nervy a hrozí ďalší pád.
-• Skúste mu nohu narovnať. – narovnávanie zlomeniny je veľmi bolestivé a môže poškodiť cievy – nechajte to záchranárom.</t>
+• Skúste mu nohu narovnať. – narovnávanie zlomeniny je veľmi bolestivé a môže poškodiť cievy. Nechajte to záchranárom.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (M, HZS).</t>
@@ -2763,7 +2763,7 @@
     <t xml:space="preserve">Leží medzi posteľou a skriňou. Je veľmi ťažký, my dvaja ho nezdvihneme. Bývame na štvrtom poschodí bez výťahu.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Skĺzol z postele.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Skĺzol z postele.
 • ★ Udrel si hlavu, stratil vedomie? → Hlavu nie, rozpráva normálne.
 • Kde presne je zranený? → Bolí ho rameno.
 • Koľko má rokov? → Šesťdesiattri.
@@ -2774,7 +2774,7 @@
 • Neskúšajte ho dvíhať sami.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Zdvihnite ho aspoň do sedu. – ťažkého pacienta treba zdvíhať s technikou a viacerými ľuďmi – inak sa zraní on aj pomáhajúci.</t>
+    <t xml:space="preserve">• Zdvihnite ho aspoň do sedu. – ťažkého pacienta treba zdvíhať s technikou a viacerými ľuďmi, inak sa zraní on aj ten, kto pomáha.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (M, HaZZ – podľa tvojho príkladu).</t>
@@ -2793,7 +2793,7 @@
     <t xml:space="preserve">Trochu, už to skoro prestalo.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ako sa to stalo – z akej výšky spadol, čím sa zranil? → Spadla z kolobežky.
+    <t xml:space="preserve">• Ako sa to stalo? Z akej výšky spadol, čím sa zranil? → Spadla z kolobežky.
 • ★ Hýbe rukami aj nohami, cíti ich? → Áno, behá.
 • Kde presne je zranený? → Koleno.
 • Koľko má rokov? → Sedem.
@@ -2808,7 +2808,7 @@
 H2 · pri ňom</t>
   </si>
   <si>
-    <t xml:space="preserve">„Asi máme všetci chrípku – bolí nás hlava a je nám zle. Svokra je taká mimo, nevie, kde je.“</t>
+    <t xml:space="preserve">„Asi máme všetci chrípku, bolí nás hlava a je nám zle. Svokra je taká mimo, nevie, kde je.“</t>
   </si>
   <si>
     <t xml:space="preserve">Svokra je zmätená a stále zaspáva. My ostatní sme pri vedomí.</t>
@@ -2831,13 +2831,13 @@
 • ★ Je tam viac ľudí, ktorým je zle? → Áno, bolí nás všetkých štyroch, aj deti. Aj pes je od rána nejaký spavý.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Všetci hneď von z bytu na čerstvý vzduch – aj so svokrou a psom.
+    <t xml:space="preserve">• Všetci hneď von z bytu na čerstvý vzduch, aj so svokrou a psom.
 • Cestou otvorte okná a dvere, ale v byte sa nezdržujte.
-• Nič nezapínajte ani nevypínajte a nefajčite – hasiči to premerajú.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Ľahnite si všetci a vyspite sa, chrípka prejde. – oxid uhoľnatý nevidno ani necítiť – v byte sa otrava zhoršuje a spánok môže skončiť bezvedomím.
-• Dajte svokre kávu, nech sa preberie. – zmätená pacientka nemusí bezpečne prehĺtať a káva otravu nelieči – treba ju dostať von.</t>
+• Nič nezapínajte ani nevypínajte a nefajčite. Hasiči byt premerajú.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ľahnite si všetci a vyspite sa, chrípka prejde. – oxid uhoľnatý nevidno ani necítiť. V byte sa otrava zhoršuje a spánok môže skončiť bezvedomím.
+• Dajte svokre kávu, nech sa preberie. – zmätená pacientka nemusí bezpečne prehĺtať a káva otravu nelieči. Treba ju dostať von.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: CO – viac ľudí s bolesťou hlavy, svokra spavá – N, dve posádky, HaZZ.</t>
@@ -2847,7 +2847,7 @@
 H2 · pri ňom</t>
   </si>
   <si>
-    <t xml:space="preserve">„Na zastávke leží asi štrnásťročné dievča, je úplne opitá.“</t>
+    <t xml:space="preserve">„Na zastávke leží asi štrnásťročné dievča, je úplne opité.“</t>
   </si>
   <si>
     <t xml:space="preserve">Keď ňou zatrasiem, niečo zamrmle, ale oči neotvorí.</t>
@@ -2869,7 +2869,7 @@
 • Prikryte ju, nech neprechladne.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte jej vypiť veľa vody. – človek, ktorý sa ťažko preberá, nevie prehĺtať – hrozí vdýchnutie.</t>
+    <t xml:space="preserve">• Dajte jej vypiť veľa vody. – človek, ktorý sa ťažko preberá, nevie prehĺtať a hrozí vdýchnutie.</t>
   </si>
   <si>
     <t xml:space="preserve">Otrava CO
@@ -2901,8 +2901,8 @@
 • Cestou von otvorte okná a dvere, ale nezdržujte sa.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ľahnite si a odpočívajte, hlava prejde. – oxid uhoľnatý nevidno ani necítiť – kto ostane dnu, môže stratiť vedomie a zomrieť.
-• Ostaňte doma a otvorte len okno v kúpeľni. – pri otrave CO treba všetkých hneď dostať von – jedno okno nestačí.</t>
+    <t xml:space="preserve">• Ľahnite si a odpočívajte, hlava prejde. – oxid uhoľnatý nevidno ani necítiť. Kto ostane dnu, môže stratiť vedomie a zomrieť.
+• Ostaňte doma a otvorte len okno v kúpeľni. – pri otrave CO treba všetkých hneď dostať von, jedno okno nestačí.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N, HaZZ). Pokyn „všetci von“ je.</t>
@@ -2937,7 +2937,7 @@
 • Ak zaspí, otočte ju na bok a sledujte dych.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vyvolajte jej zvracanie prstom. – spavý človek môže zvratky vdýchnuť – zvracanie sa nevyvoláva.
+    <t xml:space="preserve">• Vyvolajte jej zvracanie prstom. – spavý človek môže zvratky vdýchnuť. Zvracanie sa nevyvoláva.
 • Dajte jej silnú kávu, nech nezaspí. – káva neruší účinok liekov a zaťaží srdce.</t>
   </si>
   <si>
@@ -2965,7 +2965,7 @@
 • Nech zvyšky vypľuje a vypláchne si ústa, ale nič nepije.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vyvolajte zvracanie prstom v krku. – žieravina pri zvracaní poleptá pažerák druhýkrát a zvratky môžu vdýchnuť – zvracanie sa nevyvoláva.
+    <t xml:space="preserve">• Vyvolajte zvracanie prstom v krku. – žieravina pri zvracaní poleptá pažerák druhýkrát a zvratky môže vdýchnuť. Zvracanie sa nevyvoláva.
 • Dajte mu vypiť mlieko alebo olej, zneutralizuje to. – mlieko ani olej jed nezneutralizujú, iba vyvolajú zvracanie.</t>
   </si>
   <si>
@@ -3009,7 +3009,7 @@
 • Ak sa dá, nech si na ranu pritlačí vreckovku.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Odvezte ho domov, vyspí sa z toho. – úraz hlavy pod vplyvom alkoholu môže byť vážny – musí ho vyšetriť lekár.</t>
+    <t xml:space="preserve">• Odvezte ho domov, vyspí sa z toho. – úraz hlavy pod vplyvom alkoholu môže byť vážny. Musí ho vyšetriť lekár.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (M, PZ).</t>
@@ -3073,8 +3073,8 @@
 • Ak prestane reagovať alebo bude ťažko dýchať, hneď volajte znova.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Okúpte ju v studenej vode, nech zrazíte horúčku. – studený kúpeľ spôsobí triašku a zhorší prekrvenie – dieťa v šoku ho neznesie.
-• Dajte jej antibiotikum, ktoré vám ostalo od minule. – antibiotikum podáva lekár – zvyšky liekov môžu zakryť príznaky a spavé dieťa môže zvratky vdýchnuť.</t>
+    <t xml:space="preserve">• Okúpte ju v studenej vode, nech zrazíte horúčku. – studený kúpeľ spôsobí triašku a zhorší prekrvenie. Dieťa v šoku ho neznesie.
+• Dajte jej antibiotikum, ktoré vám ostalo od minule. – antibiotikum podáva lekár. Zvyšky liekov môžu zakryť príznaky a spavé dieťa môže zvratky vdýchnuť.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: horúčka, spavosť, studené končatiny, nezblednúce fľaky – N (nové kritérium N v strome Ochorenia). Overiť, či nie K.</t>
@@ -3104,7 +3104,7 @@
 • Pripravte jej lieky a zdravotnú dokumentáciu.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte jej naraz vypiť liter vody. – veľa tekutín naraz vyvolá zvracanie – po malých dúškoch.</t>
+    <t xml:space="preserve">• Dajte jej naraz vypiť liter vody. – veľa tekutín naraz vyvolá zvracanie. Treba piť po malých dúškoch.</t>
   </si>
   <si>
     <t xml:space="preserve">Upchatý katéter
@@ -3151,8 +3151,8 @@
 • Zostaňte spolu na chodníku a svieťte baterkou, nech vás nájdu.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Skráťte si cestu dole lesom mimo chodníka. – mimo chodníka sa po tme ľahko zablúdi alebo spadne – zostaňte na značke.
-• Rozdeľte sa – vy bežte dole po pomoc, ona počká. – vyčerpaný človek osamote rýchlo prechladne a ťažšie sa hľadá – zostaňte spolu.</t>
+    <t xml:space="preserve">• Skráťte si cestu dole lesom mimo chodníka. – mimo chodníka sa po tme ľahko zablúdi alebo spadne. Zostaňte na značke.
+• Rozdeľte sa: vy bežte dole po pomoc a ona počká. – vyčerpaný človek osamote rýchlo prechladne a ťažšie sa hľadá. Zostaňte spolu.</t>
   </si>
   <si>
     <t xml:space="preserve">Horúčka u dieťaťa
@@ -3205,7 +3205,7 @@
 • Dajte si do nohavičiek čistú vložku alebo uterák, nič dovnútra.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vezmite si tabletku proti bolesti. – v tehotenstve žiadne lieky bez lekára – môžu ublížiť dieťaťu.</t>
+    <t xml:space="preserve">• Vezmite si tabletku proti bolesti. – v tehotenstve sa bez lekára neberú žiadne lieky, môžu ublížiť dieťaťu.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N). Bledá, točí sa jej hlava – známky šoku; overiť, či nie K.</t>
@@ -3244,7 +3244,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Nech mama drží nohy pri sebe, kým nepríde záchranka. – pôrod sa nedá zastaviť a zadržiavanie môže ublížiť dieťaťu aj mame.
-• Keď uvidíte hlavičku, potiahnite dieťa von. – dieťa sa rodí samo – ťahanie poraní dieťa aj mamu, hlavičku treba len jemne podopierať.</t>
+• Keď uvidíte hlavičku, potiahnite dieťa von. – dieťa sa rodí samo. Ťahanie poraní dieťa aj mamu, hlavičku treba len jemne podopierať.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí (N). Pokyny podľa skriptu.</t>
@@ -3282,8 +3282,8 @@
 • Dieťa hneď osušte, položte mame na brucho a prikryte oboch.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pupočník hneď prestrihnite nožnicami. – pupočník netreba strihať – ošetrí ho posádka; nesterilný strih hrozí infekciou a krvácaním.
-• Nech dá nohy k sebe a počká na záchranku. – pôrod v behu sa nedá zastaviť – zadržiavanie hlavičky ohrozuje dieťa aj matku.</t>
+    <t xml:space="preserve">• Pupočník hneď prestrihnite nožnicami. – pupočník netreba strihať, ošetrí ho posádka. Nesterilný strih hrozí infekciou a krvácaním.
+• Nech dá nohy k sebe a počká na záchranku. – pôrod v behu sa nedá zastaviť. Zadržiavanie hlavičky ohrozuje dieťa aj matku.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistika: pôrod v behu, tretie dieťa, viditeľná hlavička – N, vedenie pôrodu, pupočník nestrihať.</t>
@@ -3427,7 +3427,7 @@
     <t xml:space="preserve">Spavý, zmätený, reaguje len na oslovenie alebo bolesť</t>
   </si>
   <si>
-    <t xml:space="preserve">Po kolapse ostal spavý alebo je nový zmätok</t>
+    <t xml:space="preserve">Po kolapse ostal spavý alebo je novo zmätený</t>
   </si>
   <si>
     <t xml:space="preserve">Kolaps u dieťaťa, seniora alebo pri srdcových ťažkostiach</t>
@@ -3958,10 +3958,10 @@
     <t xml:space="preserve">Nie, prvýkrát.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mal pred tým bolesť na hrudi alebo búšenie srdca?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mali ste pred tým bolesť na hrudi alebo búšenie srdca?</t>
+    <t xml:space="preserve">Mal predtým bolesť na hrudi alebo búšenie srdca?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mali ste predtým bolesť na hrudi alebo búšenie srdca?</t>
   </si>
   <si>
     <t xml:space="preserve">Nie, nič také.</t>
@@ -4108,7 +4108,7 @@
     <t xml:space="preserve">Je to asi len niečo zle zjedené, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">naznačuješ diagnózu – volajúci prikývne a prehliadneš náhlu príhodu.</t>
+    <t xml:space="preserve">naznačuješ diagnózu, volajúci prikývne a prehliadneš náhlu príhodu.</t>
   </si>
   <si>
     <t xml:space="preserve">Koľko má pulz? Bije srdce pravidelne?</t>
@@ -4123,10 +4123,10 @@
     <t xml:space="preserve">Liečite sa so srdcom? Mali ste infarkt alebo stent?</t>
   </si>
   <si>
-    <t xml:space="preserve">Má aj iné ťažkosti – poruchu reči, slabú ruku, zle vidí?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Máte aj iné ťažkosti – poruchu reči, slabú ruku, zle vidíte?</t>
+    <t xml:space="preserve">Má aj iné ťažkosti, napríklad poruchu reči, slabú ruku alebo zle vidí?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máte aj iné ťažkosti, napríklad poruchu reči, slabú ruku alebo zle vidíte?</t>
   </si>
   <si>
     <t xml:space="preserve">Odpadol, stratil vedomie?</t>
@@ -4186,7 +4186,7 @@
     <t xml:space="preserve">Ale nie je to porážka, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">pri mozgovej príhode rozhoduje čas – pýtaj sa na príznaky, nie na diagnózu.</t>
+    <t xml:space="preserve">pri mozgovej príhode rozhoduje čas. Pýtaj sa na príznaky, nie na diagnózu.</t>
   </si>
   <si>
     <t xml:space="preserve">Hovorí, že by si chcel ublížiť?</t>
@@ -4276,7 +4276,7 @@
     <t xml:space="preserve">Stačí si dať niečo sladké, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">pri poruche vedomia nesmie nič ústami – najprv zisti, či vie prehĺtať.</t>
+    <t xml:space="preserve">pri poruche vedomia nesmie nič ústami. Najprv zisti, či vie prehĺtať.</t>
   </si>
   <si>
     <t xml:space="preserve">Koľko je zranených?</t>
@@ -4303,7 +4303,7 @@
     <t xml:space="preserve">Hýbete rukami aj nohami, cítite ich?</t>
   </si>
   <si>
-    <t xml:space="preserve">Kde presne je – v aute, na ceste, mimo cesty?</t>
+    <t xml:space="preserve">Kde presne je? V aute, na ceste, mimo cesty?</t>
   </si>
   <si>
     <t xml:space="preserve">Na kraji cesty.</t>
@@ -4321,7 +4321,7 @@
     <t xml:space="preserve">pri nehode rozhoduje počet zranených a mechanizmus, nie dojem volajúceho.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ako sa to stalo – z akej výšky spadol, čím sa zranil?</t>
+    <t xml:space="preserve">Ako sa to stalo? Z akej výšky spadol, čím sa zranil?</t>
   </si>
   <si>
     <t xml:space="preserve">Ako sa to stalo?</t>
@@ -4336,7 +4336,7 @@
     <t xml:space="preserve">Nie je to zlomené, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">diagnózu urobí posádka – pýtaj sa na mechanizmus a hýbanie končatinami.</t>
+    <t xml:space="preserve">diagnózu urobí posádka. Pýtaj sa na mechanizmus a hýbanie končatinami.</t>
   </si>
   <si>
     <t xml:space="preserve">Čo presne a koľko užil?</t>
@@ -4369,7 +4369,7 @@
     <t xml:space="preserve">To nebude nič vážne, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">pri otrave rozhoduje čo, koľko a kedy – pýtaj sa presne.</t>
+    <t xml:space="preserve">pri otrave rozhoduje čo, koľko a kedy. Pýtaj sa presne.</t>
   </si>
   <si>
     <t xml:space="preserve">Pije a močí normálne?</t>
@@ -4384,7 +4384,7 @@
     <t xml:space="preserve">To je len chrípka, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">prehliadneš varovné príznaky – stuhnutý krk, vyrážky, spavosť.</t>
+    <t xml:space="preserve">prehliadneš varovné príznaky ako stuhnutý krk, vyrážky a spavosť.</t>
   </si>
   <si>
     <t xml:space="preserve">V ktorom je týždni? Koľké dieťa to je?</t>
@@ -4429,7 +4429,7 @@
     <t xml:space="preserve">Ešte to chvíľu potrvá, však?</t>
   </si>
   <si>
-    <t xml:space="preserve">pôrod v behu sa podcení – pýtaj sa na kontrakcie a nutkanie tlačiť.</t>
+    <t xml:space="preserve">pôrod v behu sa podcení. Pýtaj sa na kontrakcie a nutkanie tlačiť.</t>
   </si>
   <si>
     <t xml:space="preserve">Rada volajúcemu pri odkladnom hovore (O) – správne a chybné vety, povinná bezpečnostná veta</t>
@@ -4455,8 +4455,8 @@
 • Dnes už nešoférujte.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Hneď vstaňte a prejdite sa, nech sa krv rozprúdi. – po mdlobe hrozí ďalší pád – najprv sedieť alebo ležať.
-• Dajte si na posilnenie pohárik alkoholu. – alkohol rozširuje cievy a mdlobu môže zopakovať.</t>
+    <t xml:space="preserve">• Hneď vstaňte a prejdite sa, nech sa krv rozprúdi. – po mdlobe hrozí ďalší pád. Najprv treba sedieť alebo ležať.
+• Dajte si na posilnenie pohárik alkoholu. – alkohol rozširuje cievy a mdloba sa môže zopakovať.</t>
   </si>
   <si>
     <t xml:space="preserve">Kašeľ a teplota</t>
@@ -4470,7 +4470,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Choďte hneď na pohotovosť do nemocnice. – bez varovných príznakov patríte k všeobecnému lekárovi alebo na 116117.
-• Vezmite si antibiotiká, ktoré máte doma. – operátor lieky neodporúča – o liečbe rozhodne lekár.</t>
+• Vezmite si antibiotiká, ktoré máte doma. – operátor lieky neodporúča, o liečbe rozhodne lekár.</t>
   </si>
   <si>
     <t xml:space="preserve">Zastavené krvácanie z nosa</t>
@@ -4483,7 +4483,7 @@
 • Ak sa to začne znova, nech sa predkloní a stlačí si mäkkú časť nosa na desať minút.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nech si ľahne a zakloní hlavu. – pri zaklonení steká krv do hrdla – treba sa predkloniť.
+    <t xml:space="preserve">• Nech si ľahne a zakloní hlavu. – pri zaklonení steká krv do hrdla. Treba sa predkloniť.
 • Napchajte mu do nosa vatu a nechajte ju tam do rána. – vata sa prilepí a pri vyťahovaní krvácanie obnoví.</t>
   </si>
   <si>
@@ -4497,8 +4497,8 @@
 • Hýbte sa primerane, úplne sa pohybu nevyhýbajte.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Zoberte si dvojitú dávku liekov proti bolesti. – dávkovanie liekov operátor neurčuje – vyššia dávka škodí žalúdku a obličkám.
-• Ľahnite si a týždeň nevstávajte. – úplný kľud na lôžku bolesť chrbta skôr predĺži.</t>
+    <t xml:space="preserve">• Zoberte si dvojitú dávku liekov proti bolesti. – dávkovanie liekov operátor neurčuje. Vyššia dávka škodí žalúdku a obličkám.
+• Ľahnite si a týždeň nevstávajte. – úplný pokoj na lôžku bolesť chrbta skôr predĺži.</t>
   </si>
   <si>
     <t xml:space="preserve">Operátor nerozhoduje o liekoch ani dávkach.</t>
@@ -4514,14 +4514,14 @@
 • O hodinu si tlak premerajte v pokoji, v sede.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vezmite si dve tabletky naraz, nech to dobehnete. – dávkovanie liekov operátor neurčuje – dvojitá dávka môže tlak zraziť príliš.
-• Merajte si tlak každých päť minút. – časté meranie len znepokojuje – tlak sa meria v pokoji, raz za čas.</t>
+    <t xml:space="preserve">• Vezmite si dve tabletky naraz, nech to dobehnete. – dávkovanie liekov operátor neurčuje. Dvojitá dávka môže tlak zraziť príliš nízko.
+• Merajte si tlak každých päť minút. – časté meranie len znepokojuje. Tlak sa meria v pokoji, raz za čas.</t>
   </si>
   <si>
     <t xml:space="preserve">Epileptik po záchvate</t>
   </si>
   <si>
-    <t xml:space="preserve">Ak príde ďalší záchvat, záchvat bude trvať viac ako päť minút alebo sa nepreberie, volajte hneď znova.</t>
+    <t xml:space="preserve">Ak príde ďalší záchvat, ak bude trvať viac ako päť minút alebo ak sa nepreberie, volajte hneď znova.</t>
   </si>
   <si>
     <t xml:space="preserve">• Nechajte ho ležať na boku, kým sa úplne nepreberie.
@@ -4529,7 +4529,7 @@
   </si>
   <si>
     <t xml:space="preserve">• Dajte mu hneď vypiť pohár vody. – kým sa úplne nepreberie, môže vodu vdýchnuť.
-• Dajte mu niečo do úst, aby si nepohrýzol jazyk. – do úst sa nikdy nič nevkladá – hrozí udusenie a zranenie.</t>
+• Dajte mu niečo do úst, aby si nepohrýzol jazyk. – do úst sa nikdy nič nevkladá, hrozí udusenie a zranenie.</t>
   </si>
   <si>
     <t xml:space="preserve">Úzkosť</t>
@@ -4539,11 +4539,11 @@
   </si>
   <si>
     <t xml:space="preserve">• Na linke psychologickej pomoci sú nonstop a môžete tam hovoriť, ako dlho potrebujete.
-• Skúste pomaly dýchať – nádych na štyri, výdych na šesť.
+• Skúste pomaly dýchať: nádych na štyri, výdych na šesť.
 • Zavolajte sestre alebo niekomu blízkemu, nech nie ste sám.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dajte si na spanie niečo silné z lekárničky. – operátor lieky neodporúča – kombinácia liekov môže byť nebezpečná.</t>
+    <t xml:space="preserve">• Dajte si na spanie niečo silné z lekárničky. – operátor lieky neodporúča. Kombinácia liekov môže byť nebezpečná.</t>
   </si>
   <si>
     <t xml:space="preserve">Štípnutie včelou</t>
@@ -4567,7 +4567,7 @@
 • Pite vodu a o hodinu si cukor premerajte znova.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pichnite si naraz dvojitú dávku inzulínu. – dávku inzulínu operátor neurčuje – dvojitá dávka môže spôsobiť nebezpečne nízky cukor.
+    <t xml:space="preserve">• Pichnite si naraz dvojitú dávku inzulínu. – dávku inzulínu operátor neurčuje. Dvojitá dávka môže spôsobiť nebezpečne nízky cukor.
 • Vypite niečo sladké, nech sa cukor vyrovná. – pri vysokom cukre ho sladké nápoje ešte zvýšia.</t>
   </si>
   <si>
@@ -4581,8 +4581,8 @@
 • Prekryte ju čistou náplasťou alebo obväzom.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Ranu vydezinfikujte alkoholom priamo z fľaše. – alkohol v rane páli a poškodzuje tkanivo – stačí čistá voda.
-• Ranu zalepte izolepou, nech sa nešpiní. – izolepa nie je sterilná a rana sa pod ňou zapári.</t>
+    <t xml:space="preserve">• Ranu vydezinfikujte alkoholom priamo z fľaše. – alkohol v rane páli a poškodzuje tkanivo. Stačí čistá voda.
+• Ranu zalepte izolepou, nech sa nešpiní. – izolepa nie je sterilná a rana sa pod ňou zaparí.</t>
   </si>
   <si>
     <t xml:space="preserve">Horúčka u dieťaťa</t>
@@ -4595,7 +4595,7 @@
 • Ak horúčka trvá viac ako tri dni, ozvite sa detskému lekárovi alebo na 116117.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Zabaľte ho do periny, nech sa vypotí. – dieťa s horúčkou sa nemá prehrievať – teplota ešte stúpne.
+    <t xml:space="preserve">• Zabaľte ho do periny, nech sa vypotí. – dieťa s horúčkou sa nemá prehrievať, teplota by ešte stúpla.
 • Dajte mu napiť piva, to zrazí horúčku. – alkohol je pre dieťa jedovatý.</t>
   </si>
   <si>
@@ -4605,11 +4605,11 @@
     <t xml:space="preserve">Ak bude spavé, začne zvracať alebo sa bude správať inak ako zvyčajne, volajte hneď 155.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pripravte si obal od lieku a hmotnosť dieťaťa – toxikológ sa na to opýta.
+    <t xml:space="preserve">• Pripravte si obal od lieku a zistite hmotnosť dieťaťa, toxikológ sa na ne opýta.
 • Lieky odložte z dosahu detí.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Vyvolajte mu zvracanie prstom. – zvracanie sa nevyvoláva – dieťa môže vdýchnuť zvratky.
+    <t xml:space="preserve">• Vyvolajte mu zvracanie prstom. – zvracanie sa nevyvoláva, dieťa môže vdýchnuť zvratky.
 • Dajte mu vypiť mlieko, aby liek zriedilo. – mlieko pri otrave nepomáha a niektoré lieky sa s ním vstrebú rýchlejšie.</t>
   </si>
   <si>
@@ -4623,7 +4623,7 @@
 • Ak sa to opakuje každý mesiac, poraďte sa s gynekológom alebo na 116117.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Zoberte si ešte tri tabletky, nech to zaberie. – dávkovanie liekov operátor neurčuje – hrozí predávkovanie.
+    <t xml:space="preserve">• Zoberte si ešte tri tabletky, nech to zaberie. – dávkovanie liekov operátor neurčuje, hrozí predávkovanie.
 • Vypite pohárik alkoholu, uvoľní to kŕče. – alkohol s liekmi proti bolesti škodí žalúdku a pečeni.</t>
   </si>
   <si>
@@ -4651,7 +4651,7 @@
     <t xml:space="preserve">Držte telefón pri uchu a stláčajte jednou rukou.</t>
   </si>
   <si>
-    <t xml:space="preserve">s telefónom pri uchu sa nedá stláčať oboma rukami – reproduktor uvoľní ruky.</t>
+    <t xml:space="preserve">s telefónom pri uchu sa nedá stláčať oboma rukami, reproduktor uvoľní ruky.</t>
   </si>
   <si>
     <t xml:space="preserve">Doplnené podľa skriptu.</t>
@@ -4681,7 +4681,7 @@
     <t xml:space="preserve">Najprv mu hľadajte pulz na krku.</t>
   </si>
   <si>
-    <t xml:space="preserve">hľadanie pulzu laika len zdržiava – keď nedýcha normálne, stláča sa hneď.</t>
+    <t xml:space="preserve">hľadanie pulzu laika len zdržiava. Keď nedýcha normálne, stláča sa hneď.</t>
   </si>
   <si>
     <t xml:space="preserve">dospelý – 4. pokyn</t>
@@ -4693,7 +4693,7 @@
     <t xml:space="preserve">Najprv mu dvakrát vdýchnite do úst.</t>
   </si>
   <si>
-    <t xml:space="preserve">pri telefonickej resuscitácii dospelého laik iba stláča – vdychy ho zdržia.</t>
+    <t xml:space="preserve">pri telefonickej resuscitácii dospelého laik iba stláča, vdychy ho zdržia.</t>
   </si>
   <si>
     <t xml:space="preserve">Sedí. Hĺbka: skript „asi 5 cm“, hra „5 až 6 cm“ (ERC 5–6 cm).</t>
@@ -4708,7 +4708,7 @@
     <t xml:space="preserve">Najprv ho otočte hore nohami, nech z neho vytečie voda.</t>
   </si>
   <si>
-    <t xml:space="preserve">vylievanie vody stráca drahé minúty – treba hneď oživovať.</t>
+    <t xml:space="preserve">vylievanie vody stráca drahé minúty, treba hneď oživovať.</t>
   </si>
   <si>
     <t xml:space="preserve">utopený – 3. pokyn</t>
@@ -4723,7 +4723,7 @@
     <t xml:space="preserve">Len stláčajte, vdychy pri utopenom nikdy nerobte.</t>
   </si>
   <si>
-    <t xml:space="preserve">pri utopení chýba kyslík – kto vie dýchať z úst do úst, má začať 5 vdychmi.</t>
+    <t xml:space="preserve">pri utopení chýba kyslík. Kto vie dýchať z úst do úst, má začať 5 vdychmi.</t>
   </si>
   <si>
     <t xml:space="preserve">Podľa ERC (utopený: 5 úvodných vdychov).</t>
@@ -4753,7 +4753,7 @@
     <t xml:space="preserve">Tlačte dlaňou celou váhou.</t>
   </si>
   <si>
-    <t xml:space="preserve">dojča má krehký hrudník – stláča sa dvoma prstami asi do hĺbky 4 cm.</t>
+    <t xml:space="preserve">dojča má krehký hrudník, stláča sa dvoma prstami asi do hĺbky 4 cm.</t>
   </si>
   <si>
     <t xml:space="preserve">Podľa skriptu (dojča: dva prsty, ~4 cm, 5 vdychov, 15 : 2).</t>
@@ -4768,7 +4768,7 @@
     <t xml:space="preserve">Zatraste ním, nech sa preberie.</t>
   </si>
   <si>
-    <t xml:space="preserve">trasenie dojčaťa je nebezpečné a stráca čas – treba hneď stláčať.</t>
+    <t xml:space="preserve">trasenie dojčaťa je nebezpečné a stráca čas. Treba hneď stláčať.</t>
   </si>
   <si>
     <t xml:space="preserve">Tempo</t>
@@ -4861,7 +4861,7 @@
     <t xml:space="preserve">nie (zámerne chybný)</t>
   </si>
   <si>
-    <t xml:space="preserve">každé prerušenie stláčania znižuje šancu na prežitie – stláča sa bez prestávky, kým nepríde posádka.</t>
+    <t xml:space="preserve">každé prerušenie stláčania znižuje šancu na prežitie. Stláča sa bez prestávky, kým nepríde posádka.</t>
   </si>
   <si>
     <t xml:space="preserve">dospelý – 5.</t>
@@ -4888,7 +4888,7 @@
     <t xml:space="preserve">Zatraste ním, aby sa prebral.</t>
   </si>
   <si>
-    <t xml:space="preserve">trasenie dojčaťa je nebezpečné a stráca čas – treba hneď stláčať a vdychovať.</t>
+    <t xml:space="preserve">trasenie dojčaťa je nebezpečné a stráca čas. Treba hneď stláčať a vdychovať.</t>
   </si>
   <si>
     <t xml:space="preserve">dojča – 4.</t>
@@ -4897,7 +4897,7 @@
     <t xml:space="preserve">Dajte mu napiť, nech sa preberie.</t>
   </si>
   <si>
-    <t xml:space="preserve">dojča bez vedomia nevie prehĺtať – voda mu zatečie do dýchacích ciest.</t>
+    <t xml:space="preserve">dojča bez vedomia nevie prehĺtať a voda mu zatečie do dýchacích ciest.</t>
   </si>
   <si>
     <t xml:space="preserve">Kazuistiky – prerozprávané modelové prípady (detaily vymyslené) s ideálnym postupom a zdrojom</t>
@@ -4932,13 +4932,13 @@
 Utorok 21:40, Košice. Volá žena z bytu na treťom poschodí.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Adresa a čo sa stalo – Poloha je prvá – keby sa hovor prerušil, posádka vie, kam ísť.
-2. Vedomie: nereaguje ani na bolesť – Kto nereaguje, je v ohrození života – ďalšia otázka je dýchanie.
+    <t xml:space="preserve">1. Adresa a čo sa stalo – Poloha je prvá: keby sa hovor prerušil, posádka vie, kam ísť.
+2. Vedomie: nereaguje ani na bolesť – Kto nereaguje, je v ohrození života. Ďalšia otázka je dýchanie.
 3. Dýchanie: na „chrápe“ sa opýtaj „Dýcha normálne, alebo len občas zalapá?“ – Chrčanie raz za desať sekúnd nie je normálne dýchanie. Je to zástava.
 4. Náhle zastavenie obehu, stupeň K – Pri zástave sa nečaká na ďalšie podrobnosti.
 5. Posádka a lekár do 90 s
-6. TANR: na chrbát na zem, stláčanie 100 – 120-krát za minútu – Volajúca stláča, kým nepríde posádka.
-7. „Je tam ešte niekto?“ – dcéra otvorí dvere a čaká pri vchode</t>
+6. TANR: na chrbát na zem, stláčanie 100 až 120-krát za minútu – Volajúca stláča, kým nepríde posádka.
+7. „Je tam ešte niekto?“ Dcéra otvorí dvere a čaká pri vchode.</t>
   </si>
   <si>
     <t xml:space="preserve">• Laik opíše lapavé dýchanie ako chrápanie, chrčanie, vzdychanie alebo „ešte dýcha“. Vždy sa pýtaj, či dýcha normálne.
@@ -4970,10 +4970,10 @@
 4. Posádka a lekár do 90 s
 5. „Je tam ešte niekto?“ a „Je nablízku defibrilátor?“ – Keď je pri pacientovi viac ľudí, jeden stláča a druhý beží po AED.
 6. TANR a pomocník po AED – AED zapnúť a robiť, čo hovorí. Stláčanie sa prerušuje len na analýzu a výboj.
-7. TANR – tempo 100 – 120-krát za minútu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Pri jednom zachráncovi ho neposielaj po AED – stláčanie by sa prerušilo. Pri dvoch a viacerých áno.
+7. TANR v tempe 100 až 120-krát za minútu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Jediného zachráncu po AED neposielaj, stláčanie by sa prerušilo. Keď sú pri pacientovi dvaja alebo viacerí, jeden ide po AED.
 • Defibrilácia v prvých minútach zástavy výrazne zvyšuje šancu na prežitie. Operátor ju urýchli, keď sa na AED opýta.
 • Keď AED príde, nech ho zapnú a robia, čo hovorí. Operátor ostáva na linke.</t>
   </si>
@@ -4994,7 +4994,7 @@
 Pondelok 12:45, Spišská Nová Ves. Volá vnučka, ktorá je na návšteve u starej mamy.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Adresa a čo sa stalo – Volajúca chce čakať do rána – o naliehavosti však rozhoduje operátor.
+    <t xml:space="preserve">1. Adresa a čo sa stalo – Volajúca chce čakať do rána, o naliehavosti však rozhoduje operátor.
 2. Vedomie a dýchanie sú v poriadku
 3. Neurológia: ovisnutý kútik, slabá ruka, porucha reči? – Stačí jeden z príznakov.
 4. „Kedy bola naposledy v poriadku?“ – Od toho závisí, či sa dá cielená liečba ešte podať.
@@ -5023,17 +5023,17 @@
 Štvrtok 9:15, Michalovce. Volá sama pacientka z domu.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Kto volá: H1 – pacientka sama – Vedomie je zrejmé z rozhovoru. Pýtaj sa na dýchanie a farbu kože.
+    <t xml:space="preserve">1. Kto volá: H1, pacientka sama – Vedomie je zrejmé z rozhovoru. Pýtaj sa na dýchanie a farbu kože.
 2. Koža: bledá, studený pot; aj dýchavica
-3. Kategória Kardiologické ťažkosti, nie bolesť brucha – Pálenie pod hrudnou kosťou so studeným potom je podozrenie na infarkt, aj keď to volajúca volá žalúdok.
-4. „Kde presne to bolí a kam to vystreľuje?“ – medzi lopatky a do sánky
+3. Kategória Kardiologické ťažkosti, nie bolesť brucha – Pálenie pod hrudnou kosťou so studeným potom je podozrenie na infarkt, aj keď ho volajúca považuje za žalúdok.
+4. „Kde presne to bolí a kam to vystreľuje?“ Medzi lopatky a do sánky.
 5. Stupeň K, posádka a lekár do 90 s
 6. Pokyny: pokoj, sadnúť si, odomknúť, pripraviť lieky</t>
   </si>
   <si>
     <t xml:space="preserve">• Ženy, starší ľudia a diabetici mávajú pri infarkte netypické príznaky: nevoľnosť, pálenie „žáhy“, únavu, bolesť medzi lopatkami.
 • V dánskej štúdii dostali pacienti s infarktom a netypickými príznakmi záchranku zriedkavejšie a mali vyššiu úmrtnosť.
-• Diagnózu „žalúdok“ od volajúceho nepreberaj – pýtaj sa na príznaky.</t>
+• Diagnózu „žalúdok“ od volajúceho nepreberaj. Pýtaj sa na príznaky.</t>
   </si>
   <si>
     <t xml:space="preserve">Netypické príznaky infarktu a menej výjazdov (Healio, dánska štúdia 2021) – https://www.healio.com/news/cardiology/20210614/atypical-mi-symptoms-tied-to-negative-outcomes-lower-odds-of-emergency-response</t>
@@ -5050,16 +5050,16 @@
 Utorok 16:30, Trebišov. Volá žena zo záhrady.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Kto volá: H1 – pacientka sama
+    <t xml:space="preserve">1. Kto volá: H1, pacientka sama
 2. Dýchanie: piští pri nádychu, ťažko hovorí – Chrapot a pískanie sú varovné.
 3. Alergia: opuch pier a jazyka, nepovie celú vetu
 4. Stupeň N, posádka do 90 s
-5. „Máte adrenalínové pero?“ – a naviesť ju – Strach z pera je častý. Poistka, vonkajšia strana stehna, aj cez oblečenie, podržať.
+5. „Máte adrenalínové pero?“ Potom ju naviesť. – Strach z pera je častý. Poistka, vonkajšia strana stehna, aj cez oblečenie, podržať.
 6. Sedieť, pri slabosti ľahnúť s nohami hore, nevstávať</t>
   </si>
   <si>
     <t xml:space="preserve">• Adrenalín do svalu je pri anafylaxii prvý liek. Čakanie na posádku pacienta ohrozuje.
-• Pacient s anafylaxiou nemá vstávať ani chodiť – hrozí náhly kolaps.
+• Pacient s anafylaxiou nemá vstávať ani chodiť, hrozí náhly kolaps.
 • Ak sa stav po 5 až 15 minútach nezlepší a je k dispozícii druhé pero, podáva sa druhá dávka.</t>
   </si>
   <si>
@@ -5079,7 +5079,7 @@
   <si>
     <t xml:space="preserve">1. Adresa a čo sa stalo
 2. Pôrod: týždeň a koľké dieťa – Tretie dieťa rodí rýchlejšie.
-3. Kontrakcie a nutkanie tlačiť – vidno hlavičku – Viditeľná hlavička = pôrod v behu, nikam sa necestuje.
+3. Kontrakcie a nutkanie tlačiť: vidno hlavičku – Viditeľná hlavička = pôrod v behu, nikam sa necestuje.
 4. Stupeň N, posádka do 90 s
 5. Viesť pôrod: poloha, uteráky, hlavičku neťahať ani nezadržiavať
 6. Po pôrode: osušiť, na brucho matky, prikryť; pupočník nestrihať</t>
@@ -5104,17 +5104,17 @@
 Nedeľa 5:00, Rožňava. Volá mama trojročného dievčatka.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Adresa a čo sa stalo – Mama sa pýta na pediatra – vyzerá to na radu.
+    <t xml:space="preserve">1. Adresa a čo sa stalo – Mama sa pýta na pediatra, vyzerá to na radu.
 2. Vedomie: stále zaspáva – Spavé dieťa s horúčkou nie je odkladný hovor.
 3. Koža: bledá, studené ruky a nohy
-4. „Má vyrážky, stuhnutý krk, je spavá?“ – fľaky pod pohárom nezblednú – Môže ísť o sepsu.
-5. „Pije a močí?“ – suchá plienka
-6. Stupeň N, posádka do 90 s – nie rada ani 116117</t>
+4. „Má vyrážky, stuhnutý krk, je spavá?“ Fľaky pod pohárom nezblednú. – Môže ísť o sepsu.
+5. „Pije a močí?“ Plienka je suchá.
+6. Stupeň N a posádka do 90 s, žiadna rada ani 116117</t>
   </si>
   <si>
     <t xml:space="preserve">• Horúčka u čulého dieťaťa, ktoré pije, je odkladná. Spavé dieťa s fľakmi alebo so studenými končatinami nie.
 • Skúška pohárom: fľaky, ktoré pri pritlačení pohára nezblednú, sú dôvod na okamžitú pomoc. Na tmavšej koži ich hľadaj na dlaniach, chodidlách a v spojovkách.
-• Vyrážka býva neskorý príznak – pri spavom dieťati sa na ňu nečaká.</t>
+• Vyrážka býva neskorý príznak. Pri spavom dieťati sa na ňu nečaká.</t>
   </si>
   <si>
     <t xml:space="preserve">Royal Children's Hospital Melbourne – Fever and petechiae/purpura – https://www.rch.org.au/clinicalguide/guideline_index/fever_and_petechiae_purpura/</t>
@@ -5133,15 +5133,15 @@
   <si>
     <t xml:space="preserve">1. Adresa a čo sa stalo – Volajúci si myslí, že ide o chrípku.
 2. Vedomie: svokra je zmätená a spavá – Porucha vedomia mení naliehavosť.
-3. „Je tam viac ľudí, ktorým je zle?“ – všetci štyria aj pes – Rovnaké ťažkosti u viacerých naraz, bez horúčky = mysli na oxid uhoľnatý.
-4. „Je k nim prístup, nehrozí tam niečo?“ – celú noc kúrili v piecke
+3. „Je tam viac ľudí, ktorým je zle?“ Všetci štyria aj pes. – Rovnaké ťažkosti u viacerých naraz, bez horúčky = mysli na oxid uhoľnatý.
+4. „Je k nim prístup, nehrozí tam niečo?“ Celú noc kúrili v piecke.
 5. Intoxikácia, stupeň N, dve posádky
 6. Súčinnosť: hasiči zmerajú CO a vyvetrajú
 7. Pokyny: všetci von, nič nezapínať – Kým sa byt nevyvetrá, je nebezpečný aj pre záchranárov.</t>
   </si>
   <si>
     <t xml:space="preserve">• Bolesť hlavy, nevoľnosť a spavosť u celej rodiny naraz, najmä v zime pri kúrení, je typická pre otravu oxidom uhoľnatým.
-• Prvý pokyn je dostať všetkých von – nie liečiť doma.
+• Prvý pokyn je dostať všetkých von.
 • Pri podozrení na CO vždy požiadaj o hasičov.</t>
   </si>
   <si>
@@ -5159,10 +5159,10 @@
 Piatok 14:10, Moldava nad Bodvou. Volá syn.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Adresa a čo sa stalo – volajúci hovorí o porážke
+    <t xml:space="preserve">1. Adresa a čo sa stalo. Volajúci hovorí o porážke.
 2. Vedomie: zmätený; koža: bledý, spotený – Studený pot pri zmätenosti je typický pre nízky cukor.
-3. „Máte glukomer? Koľko ukazuje?“ – 2,1 – V rodine diabetika býva glukomer takmer vždy – stačí sa opýtať.
-4. „Pichal si inzulín? Jedol?“ – inzulín bez obeda
+3. „Máte glukomer? Koľko ukazuje?“ Ukazuje 2,1. – V rodine diabetika býva glukomer takmer vždy, stačí sa opýtať.
+4. „Pichal si inzulín? Jedol?“ Inzulín si pichol, obed vynechal.
 5. „Vie prehĺtať?“ – Sladké len vtedy, keď je pri vedomí a bezpečne prehĺta.
 6. Stupeň N, posádka do 90 s
 7. Pokyny: sladký nápoj, sedieť; keby prestal reagovať, nič do úst a na bok</t>
@@ -5170,7 +5170,7 @@
   <si>
     <t xml:space="preserve">• Nízky cukor je najčastejšia zameniteľná „porážka“ a overíš ho jednou otázkou na glukomer.
 • Sladké len pri vedomí a bezpečnom prehĺtaní.
-• Aj keď sa po sladkom zlepší, posádku neruš – pri inzulíne môže cukor znova klesnúť.</t>
+• Aj keď sa po sladkom zlepší, posádku neruš. Pri inzulíne môže cukor znova klesnúť.</t>
   </si>
   <si>
     <t xml:space="preserve">JEMS – The Stroke That Wasn't – https://www.jems.com/?p=222438
@@ -5196,7 +5196,7 @@
 6. Pokyny: prilbu nesnímať, nehýbať ním, tlak na krvácanie, zabezpečiť miesto</t>
   </si>
   <si>
-    <t xml:space="preserve">• Mechanizmus (rýchlosť, vymrštenie z vozidla) je kritérium samo osebe – aj keď pacient „len“ hovorí z cesty.
+    <t xml:space="preserve">• Mechanizmus úrazu (rýchlosť, vymrštenie z vozidla) je kritérium samo osebe, aj keď pacient „len“ hovorí z cesty.
 • Prilba sa sníma len vtedy, keď pacient nedýcha a treba ho oživovať.
 • Bezpečnosť na mieste: výstražný trojuholník, svetlá, ľudia mimo cesty.</t>
   </si>
@@ -5234,10 +5234,10 @@
 Isté známky smrti (O)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nereaguje a nedýcha normálne – aj občasné lapavé dychy sú zástava. Hneď TANR.
-• Bezvedomie s normálnym dýchaním je K, ale bez TANR – stabilizovaná poloha.
+    <t xml:space="preserve">• Nereaguje a nedýcha normálne: aj občasné lapavé dychy sú zástava. Hneď TANR.
+• Bezvedomie s normálnym dýchaním je K, ale bez TANR. Pacient patrí do stabilizovanej polohy.
 • Krátky kolaps, po ktorom je úplne v poriadku, je M; senior, dieťa alebo srdcové ťažkosti robia z kolapsu N.
-• Isté známky smrti (stuhnutý, studený, fialové škvrny) – bez výjazdu, prehliadka mŕtveho tela.</t>
+• Isté známky smrti (stuhnutý, studený, fialové škvrny) znamenajú hovor bez výjazdu a prehliadku mŕtveho tela.</t>
   </si>
   <si>
     <t xml:space="preserve">Dýchanie a alergia</t>
@@ -5252,10 +5252,10 @@
 Kašeľ a teplota (O)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nevie povedať celú vetu, modré pery alebo vdýchnuté sústo – K.
-• Opuch tváre a jazyka po bodnutí či lieku – N a hneď adrenalínové pero.
-• Rýchle dýchanie po rozrušení s mravčením okolo úst je M – vylúč bolesť na hrudi.
-• Kašeľ bez dýchavice je O – rada alebo 116117.</t>
+    <t xml:space="preserve">• Keď nevie povedať celú vetu, má modré pery alebo vdýchol sústo, je to K.
+• Opuch tváre a jazyka po bodnutí či lieku je N. Hneď nech použije adrenalínové pero.
+• Rýchle dýchanie po rozrušení s mravčením okolo úst je M, ale najprv vylúč bolesť na hrudi.
+• Kašeľ bez dýchavice je O: rada alebo 116117.</t>
   </si>
   <si>
     <t xml:space="preserve">Srdce a bolesť</t>
@@ -5270,10 +5270,10 @@
 Zabudnutá tabletka na tlak (O)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Bolesť na hrudi s bledosťou, potom a dýchavicou je K – posádka a lekár.
+    <t xml:space="preserve">• Bolesť na hrudi s bledosťou, potom a dýchavicou je K, ide posádka aj lekár.
 • Náhla prudká bolesť bez úrazu je N.
 • Vysoký tlak bez ďalších ťažkostí je M; s poruchou reči, slabosťou ruky či bolesťou na hrudi je to iný problém.
-• Otázky na liečbu sú O – operátor nerozhoduje o liekoch ani dávkach.</t>
+• Otázky na liečbu sú O. Operátor nerozhoduje o liekoch ani dávkach.</t>
   </si>
   <si>
     <t xml:space="preserve">Neurológia a diabetes</t>
@@ -5288,10 +5288,10 @@
 Nízky cukor (M)</t>
   </si>
   <si>
-    <t xml:space="preserve">• FAST – ovisnutý kútik, slabá ruka, porucha reči – N a zisti, kedy bol naposledy v poriadku.
+    <t xml:space="preserve">• Ovisnutý kútik, slabá ruka alebo porucha reči (FAST) sú N. Zisti, kedy bol pacient naposledy v poriadku.
 • Kŕče, ktoré neprestávajú alebo sa opakujú, sú K.
 • Zmätený diabetik je N; sladké len vtedy, keď vie prehĺtať.
-• Nízky cukor u orientovaného diabetika je M – nech zje niečo sladké.</t>
+• Nízky cukor u orientovaného diabetika je M, nech zje niečo sladké.</t>
   </si>
   <si>
     <t xml:space="preserve">Úrazy a dopravné nehody</t>
@@ -5307,9 +5307,9 @@
   </si>
   <si>
     <t xml:space="preserve">• Bezvedomie po úraze, pád z výšky, bodná rana na trupe či veľké krvácanie sú K.
-• Závažný mechanizmus nehody – vysoká rýchlosť, zakliesnenie, motorkár – je N; hasiči na vyslobodenie, polícia k nehode.
+• Závažný mechanizmus nehody (vysoká rýchlosť, zakliesnenie, motorkár) je N. Hasiči idú na vyslobodenie, polícia k nehode.
 • Senior po páde, ktorý nevie vstať, ale je pri vedomí, je M.
-• Odreniny a drobné rany sú O – rada.</t>
+• Odreniny a drobné rany sú O, stačí rada.</t>
   </si>
   <si>
     <t xml:space="preserve">Intoxikácie a psychické ťažkosti</t>
@@ -5325,9 +5325,9 @@
   </si>
   <si>
     <t xml:space="preserve">• Lieky na spanie či na depresiu, vysoká dávka a spavosť sú N.
-• Hrozba samovraždy s bezprostredným rizikom je N – vyžiadaj PZ, pri balkóne aj hasičov.
-• Dieťa, ktoré mohlo vypiť chemikáliu, je M – nevyvolávať zvracanie.
-• Úzkosť bez myšlienok na ublíženie si je O – linka psychologickej pomoci.</t>
+• Hrozba samovraždy s bezprostredným rizikom je N. Vyžiadaj PZ, pri balkóne aj hasičov.
+• Dieťa, ktoré mohlo vypiť chemikáliu, je M. Zvracanie nevyvolávať.
+• Úzkosť bez myšlienok na ublíženie si je O, odporuč linku psychologickej pomoci.</t>
   </si>
   <si>
     <t xml:space="preserve">Pôrod, gynekológia a krvácanie</t>
@@ -5342,7 +5342,7 @@
 Menštruačné bolesti (O)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Nutkanie tlačiť alebo viditeľná hlavička – N a veď pôrod telefonicky.
+    <t xml:space="preserve">• Nutkanie tlačiť alebo viditeľná hlavička je N. Veď pôrod telefonicky.
 • Silné krvácanie v tehotenstve je N.
 • Zvracanie krvi alebo čierna stolica je N; pri šoku hrozí zhoršenie.
 • Menštruačné bolesti bez silného krvácania sú O.</t>
@@ -5360,10 +5360,10 @@
 Otec volal, že ho bolí hrudník (K)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Horúčka u čulého dieťaťa, ktoré pije, je O – ale opýtaj sa na vyrážky, stuhnutý krk a spavosť.
+    <t xml:space="preserve">• Horúčka u čulého dieťaťa, ktoré pije, je O. Opýtaj sa však na vyrážky, stuhnutý krk a spavosť.
 • Dehydratácia so zmätenosťou u seniorky je M.
-• Túlavý pes je vec pre 112 – odovzdaj hovor.
-• Opýtaj sa vždy „Ste pri pacientovi?“ – volajúci, ktorý nie je pri pacientovi, odpovedá z pamäti.</t>
+• Túlavý pes je vec pre 112, odovzdaj hovor.
+• Vždy sa opýtaj: „Ste pri pacientovi?“ Volajúci, ktorý pri ňom nie je, odpovedá z pamäti.</t>
   </si>
   <si>
     <t xml:space="preserve">AED na mape (polohy sú ilustračné)</t>

</xml_diff>